<commit_message>
Add travel time information about former car users and remaining pt users
</commit_message>
<xml_diff>
--- a/src/main/R/results-analysis_Siemensbahn.xlsx
+++ b/src/main/R/results-analysis_Siemensbahn.xlsx
@@ -433,11 +433,14 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>SiBa_v1</t>
+          <t>Siemensbahn+v1</t>
         </is>
       </c>
       <c r="B4">
         <v>577042817.9558327</v>
+      </c>
+      <c r="C4">
+        <v>27915089.2804002</v>
       </c>
       <c r="D4">
         <v>277436.0786111111</v>
@@ -452,11 +455,14 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>SiBa_v2</t>
+          <t>Siemensbahn+v2</t>
         </is>
       </c>
       <c r="B5">
         <v>576954629.6421262</v>
+      </c>
+      <c r="C5">
+        <v>27805258.96553729</v>
       </c>
       <c r="D5">
         <v>277845.8266666667</v>

</xml_diff>

<commit_message>
Sample upscale corrected for all total results
</commit_message>
<xml_diff>
--- a/src/main/R/results-analysis_Siemensbahn.xlsx
+++ b/src/main/R/results-analysis_Siemensbahn.xlsx
@@ -351,7 +351,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F5"/>
+  <dimension ref="A1:E5"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
@@ -362,25 +362,20 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>Total Monetized Score [EUR/day]</t>
+          <t>Total Monetized Score Delimited Region [EUR/day]</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>Total Monetized Score Delimited Region [EUR/day]</t>
+          <t>Total Travel Time for PT-Users [h/day]</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>Total Travel Time for PT-Users [h/day]</t>
+          <t>Total Transfers [1/day]</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>Total Transfers [1/day]</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Total Car-km [km/day]</t>
         </is>
@@ -393,19 +388,16 @@
         </is>
       </c>
       <c r="B2">
-        <v>577758076.2797799</v>
+        <v>21122548.0872282</v>
       </c>
       <c r="C2">
-        <v>21808131.96895123</v>
+        <v>138136.0972222222</v>
       </c>
       <c r="D2">
-        <v>276979.0491666667</v>
+        <v>153750</v>
       </c>
       <c r="E2">
-        <v>266913</v>
-      </c>
-      <c r="F2">
-        <v>4514604.345</v>
+        <v>1979394.16</v>
       </c>
     </row>
     <row r="3">
@@ -415,19 +407,16 @@
         </is>
       </c>
       <c r="B3">
-        <v>577686297.2583973</v>
+        <v>21133550.90304748</v>
       </c>
       <c r="C3">
-        <v>21827838.55077017</v>
+        <v>140969.8083333333</v>
       </c>
       <c r="D3">
-        <v>277538.0641666666</v>
+        <v>152430</v>
       </c>
       <c r="E3">
-        <v>266953</v>
-      </c>
-      <c r="F3">
-        <v>4508901.715</v>
+        <v>1941973.24</v>
       </c>
     </row>
     <row r="4">
@@ -437,19 +426,16 @@
         </is>
       </c>
       <c r="B4">
-        <v>577792258.8360479</v>
+        <v>21156219.49181719</v>
       </c>
       <c r="C4">
-        <v>21847699.31854214</v>
+        <v>142385.475</v>
       </c>
       <c r="D4">
-        <v>277636.7913888889</v>
+        <v>149870</v>
       </c>
       <c r="E4">
-        <v>266886</v>
-      </c>
-      <c r="F4">
-        <v>4507408.865</v>
+        <v>1911768.38</v>
       </c>
     </row>
     <row r="5">
@@ -459,19 +445,16 @@
         </is>
       </c>
       <c r="B5">
-        <v>577830827.1462517</v>
+        <v>21147884.81078412</v>
       </c>
       <c r="C5">
-        <v>21844314.12200892</v>
+        <v>142601.1638888889</v>
       </c>
       <c r="D5">
-        <v>277445.6319444444</v>
+        <v>149800</v>
       </c>
       <c r="E5">
-        <v>266531</v>
-      </c>
-      <c r="F5">
-        <v>4513263.796</v>
+        <v>1914024.07</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Travel Distance PT added
</commit_message>
<xml_diff>
--- a/src/main/R/results-analysis_Siemensbahn.xlsx
+++ b/src/main/R/results-analysis_Siemensbahn.xlsx
@@ -351,7 +351,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E5"/>
+  <dimension ref="A1:F5"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
@@ -372,10 +372,15 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
+          <t>Total Travel Distance for PT-Users [km/day]</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
           <t>Total Transfers [1/day]</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Total Car-km [km/day]</t>
         </is>
@@ -394,9 +399,12 @@
         <v>138136.0972222222</v>
       </c>
       <c r="D2">
+        <v>2256073.41</v>
+      </c>
+      <c r="E2">
         <v>153750</v>
       </c>
-      <c r="E2">
+      <c r="F2">
         <v>1979394.16</v>
       </c>
     </row>
@@ -413,9 +421,12 @@
         <v>140969.8083333333</v>
       </c>
       <c r="D3">
+        <v>2316893.95</v>
+      </c>
+      <c r="E3">
         <v>152430</v>
       </c>
-      <c r="E3">
+      <c r="F3">
         <v>1941973.24</v>
       </c>
     </row>
@@ -432,9 +443,12 @@
         <v>142385.475</v>
       </c>
       <c r="D4">
+        <v>2344499.19</v>
+      </c>
+      <c r="E4">
         <v>149870</v>
       </c>
-      <c r="E4">
+      <c r="F4">
         <v>1911768.38</v>
       </c>
     </row>
@@ -451,9 +465,12 @@
         <v>142601.1638888889</v>
       </c>
       <c r="D5">
+        <v>2338632.79</v>
+      </c>
+      <c r="E5">
         <v>149800</v>
       </c>
-      <c r="E5">
+      <c r="F5">
         <v>1914024.07</v>
       </c>
     </row>

</xml_diff>